<commit_message>
feat: JAM66D45-625/LB al catálogo (fila 62) + herramienta agregar_panel.py con auto-detección venv
</commit_message>
<xml_diff>
--- a/bipv_python/datos/paneles_catalogo.xlsx
+++ b/bipv_python/datos/paneles_catalogo.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V61"/>
+  <dimension ref="A1:V62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5131,6 +5131,79 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>JA Solar</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>JA Solar JAM66D45-625/LB</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>625</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2382x1134x30</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>45</v>
+      </c>
+      <c r="H62" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Ficha técnica oficial JAM66D45-625/LB. Alpha_Isc=+0.045%/°C. Bifacial 80%±5%. Peso=33.1kg. Vmax=1500V. IEC61215/61730.</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>N-Type Bifacial</t>
+        </is>
+      </c>
+      <c r="L62" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="M62" t="n">
+        <v>40.45</v>
+      </c>
+      <c r="N62" t="n">
+        <v>16.15</v>
+      </c>
+      <c r="O62" t="n">
+        <v>15.45</v>
+      </c>
+      <c r="P62" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>132</v>
+      </c>
+      <c r="R62" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="S62" t="n">
+        <v>171.6</v>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>Ficha oficial JA Solar JAM66D45 LB Deep Blue 4.0</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
feat: EINNOVA ESM-320 Luminous PV Bifacial al catálogo (fila 63) — BIPV τ=45%
</commit_message>
<xml_diff>
--- a/bipv_python/datos/paneles_catalogo.xlsx
+++ b/bipv_python/datos/paneles_catalogo.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V62"/>
+  <dimension ref="A1:V63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5204,6 +5204,79 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>EINNOVA Solarline</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>EINNOVA ESM-320 Luminous PV Bifacial</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>320</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2088x1128x5</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>45</v>
+      </c>
+      <c r="H63" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="I63" t="n">
+        <v>45</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Panel BIPV semi-transparente τ=45%. Frameless doble vidrio 2+2mm. Mono half-cell 182mm. Alpha_Isc=+0.045%/°C. Vmax=700Vdc IEC/UL. Certificado IEC61215/61730. 30 años garantía. einnova-solarline.com</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Mono PERC Bifacial BIPV</t>
+        </is>
+      </c>
+      <c r="L63" t="n">
+        <v>28.12</v>
+      </c>
+      <c r="M63" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="N63" t="n">
+        <v>13.77</v>
+      </c>
+      <c r="O63" t="n">
+        <v>13.01</v>
+      </c>
+      <c r="P63" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>80</v>
+      </c>
+      <c r="R63" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="S63" t="n">
+        <v>104</v>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-32 Luminous PV — 2x40 half-cells 182mm</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
feat: EINNOVA ESM-620M TopCon N-Type Black al catálogo (fila 64) — dims estimadas
</commit_message>
<xml_diff>
--- a/bipv_python/datos/paneles_catalogo.xlsx
+++ b/bipv_python/datos/paneles_catalogo.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V63"/>
+  <dimension ref="A1:V64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5277,6 +5277,79 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>EINNOVA Solarline</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>EINNOVA ESM-620M TopCon N-Type Black</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>620</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2278x1134x30</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>45</v>
+      </c>
+      <c r="H64" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Datos eléctricos: ficha oficial EINNOVA ESM-620M TopCon N-Type Black. Alpha_Isc=+0.046%/°C. Vmax=1500Vdc. Eficiencia=23.99%. DIMENSIONES ESTIMADAS (2278x1134) — confirmar con EINNOVA. Precio pendiente.</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>N-Type TopCon Mono</t>
+        </is>
+      </c>
+      <c r="L64" t="n">
+        <v>52.26</v>
+      </c>
+      <c r="M64" t="n">
+        <v>43.34</v>
+      </c>
+      <c r="N64" t="n">
+        <v>14.88</v>
+      </c>
+      <c r="O64" t="n">
+        <v>14.31</v>
+      </c>
+      <c r="P64" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>132</v>
+      </c>
+      <c r="R64" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="S64" t="n">
+        <v>171.6</v>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>Ficha EINNOVA ESM-620M — Ns y dims estimados (confirmar con fabricante)</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
fix: ESM-620M dims confirmadas 2279x1134x30mm, célula 183.75mm, Confianza=Alta
</commit_message>
<xml_diff>
--- a/bipv_python/datos/paneles_catalogo.xlsx
+++ b/bipv_python/datos/paneles_catalogo.xlsx
@@ -5293,7 +5293,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>2278x1134x30</t>
+          <t>2279x1134x30</t>
         </is>
       </c>
       <c r="G64" t="n">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Datos eléctricos: ficha oficial EINNOVA ESM-620M TopCon N-Type Black. Alpha_Isc=+0.046%/°C. Vmax=1500Vdc. Eficiencia=23.99%. DIMENSIONES ESTIMADAS (2278x1134) — confirmar con EINNOVA. Precio pendiente.</t>
+          <t>Datos eléctricos y mecánicos: ficha oficial EINNOVA ESM-620M TopCon N-Type Black. Dims confirmadas: 2279×1134×30mm. Célula 183.75×183.75mm monocristalino N-Type. Alpha_Isc=+0.046%/°C. Vmax=1500Vdc. Eficiencia=23.99%. Precio pendiente.</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -5341,12 +5341,12 @@
       </c>
       <c r="U64" t="inlineStr">
         <is>
-          <t>Ficha EINNOVA ESM-620M — Ns y dims estimados (confirmar con fabricante)</t>
+          <t>Ficha EINNOVA ESM-620M — célula 183.75×183.75mm MonoC N-Type</t>
         </is>
       </c>
       <c r="V64" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: EINNOVA ESM-530T a 550T TopCon Bifacial — 5 modelos al catálogo (filas 65-69)
</commit_message>
<xml_diff>
--- a/bipv_python/datos/paneles_catalogo.xlsx
+++ b/bipv_python/datos/paneles_catalogo.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V64"/>
+  <dimension ref="A1:V69"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5350,6 +5350,371 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>EINNOVA Solarline</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>EINNOVA ESM-530T TopCon Bifacial</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>530</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2094x1134x30</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>45</v>
+      </c>
+      <c r="H65" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-530T TopCon Bifacial. Efic=22.32%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims ESTIMADAS — confirmar con EINNOVA.</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>N-Type TopCon Bifacial Mono</t>
+        </is>
+      </c>
+      <c r="L65" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="M65" t="n">
+        <v>39</v>
+      </c>
+      <c r="N65" t="n">
+        <v>14.27</v>
+      </c>
+      <c r="O65" t="n">
+        <v>13.59</v>
+      </c>
+      <c r="P65" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>132</v>
+      </c>
+      <c r="R65" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="S65" t="n">
+        <v>171.6</v>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-T series — Ns estimado (confirmar dims)</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>EINNOVA Solarline</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>EINNOVA ESM-535T TopCon Bifacial</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>535</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2094x1134x30</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>45</v>
+      </c>
+      <c r="H66" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-535T TopCon Bifacial. Efic=22.52%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims ESTIMADAS — confirmar con EINNOVA.</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>N-Type TopCon Bifacial Mono</t>
+        </is>
+      </c>
+      <c r="L66" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="M66" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="N66" t="n">
+        <v>14.31</v>
+      </c>
+      <c r="O66" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="P66" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>132</v>
+      </c>
+      <c r="R66" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="S66" t="n">
+        <v>171.6</v>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-T series — Ns estimado (confirmar dims)</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>EINNOVA Solarline</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>EINNOVA ESM-540T TopCon Bifacial</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>540</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2094x1134x30</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>45</v>
+      </c>
+      <c r="H67" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-540T TopCon Bifacial. Efic=22.74%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims ESTIMADAS — confirmar con EINNOVA.</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>N-Type TopCon Bifacial Mono</t>
+        </is>
+      </c>
+      <c r="L67" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="M67" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="N67" t="n">
+        <v>14.35</v>
+      </c>
+      <c r="O67" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="P67" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>132</v>
+      </c>
+      <c r="R67" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="S67" t="n">
+        <v>171.6</v>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-T series — Ns estimado (confirmar dims)</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>EINNOVA Solarline</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>EINNOVA ESM-545T TopCon Bifacial</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>545</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2094x1134x30</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>45</v>
+      </c>
+      <c r="H68" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-545T TopCon Bifacial. Efic=22.95%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims ESTIMADAS — confirmar con EINNOVA.</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>N-Type TopCon Bifacial Mono</t>
+        </is>
+      </c>
+      <c r="L68" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="M68" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="N68" t="n">
+        <v>14.39</v>
+      </c>
+      <c r="O68" t="n">
+        <v>13.76</v>
+      </c>
+      <c r="P68" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>132</v>
+      </c>
+      <c r="R68" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="S68" t="n">
+        <v>171.6</v>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-T series — Ns estimado (confirmar dims)</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>EINNOVA Solarline</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>EINNOVA ESM-550T TopCon Bifacial</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>550</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>2094x1134x30</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>45</v>
+      </c>
+      <c r="H69" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-550T TopCon Bifacial. Efic=23.16%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims ESTIMADAS — confirmar con EINNOVA.</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>N-Type TopCon Bifacial Mono</t>
+        </is>
+      </c>
+      <c r="L69" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="M69" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="N69" t="n">
+        <v>14.43</v>
+      </c>
+      <c r="O69" t="n">
+        <v>13.81</v>
+      </c>
+      <c r="P69" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>132</v>
+      </c>
+      <c r="R69" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="S69" t="n">
+        <v>171.6</v>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-T series — Ns estimado (confirmar dims)</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
fix: ESM-530T a 550T dims confirmadas 2094×1134×30mm, 132 celdas 6×22, Confianza=Alta
</commit_message>
<xml_diff>
--- a/bipv_python/datos/paneles_catalogo.xlsx
+++ b/bipv_python/datos/paneles_catalogo.xlsx
@@ -5380,7 +5380,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Ficha oficial EINNOVA ESM-530T TopCon Bifacial. Efic=22.32%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims ESTIMADAS — confirmar con EINNOVA.</t>
+          <t>Ficha oficial EINNOVA ESM-530T TopCon Bifacial. Efic=22.32%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims CONFIRMADAS: 2094×1134×30mm. 132 semicélulas 6×22.</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -5414,12 +5414,12 @@
       </c>
       <c r="U65" t="inlineStr">
         <is>
-          <t>Ficha oficial EINNOVA ESM-T series — Ns estimado (confirmar dims)</t>
+          <t>Ficha oficial EINNOVA ESM-T — 132 piezas (6×22) confirmadas</t>
         </is>
       </c>
       <c r="V65" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>
@@ -5453,7 +5453,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Ficha oficial EINNOVA ESM-535T TopCon Bifacial. Efic=22.52%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims ESTIMADAS — confirmar con EINNOVA.</t>
+          <t>Ficha oficial EINNOVA ESM-535T TopCon Bifacial. Efic=22.52%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims CONFIRMADAS: 2094×1134×30mm. 132 semicélulas 6×22.</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -5487,12 +5487,12 @@
       </c>
       <c r="U66" t="inlineStr">
         <is>
-          <t>Ficha oficial EINNOVA ESM-T series — Ns estimado (confirmar dims)</t>
+          <t>Ficha oficial EINNOVA ESM-T — 132 piezas (6×22) confirmadas</t>
         </is>
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>
@@ -5526,7 +5526,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Ficha oficial EINNOVA ESM-540T TopCon Bifacial. Efic=22.74%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims ESTIMADAS — confirmar con EINNOVA.</t>
+          <t>Ficha oficial EINNOVA ESM-540T TopCon Bifacial. Efic=22.74%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims CONFIRMADAS: 2094×1134×30mm. 132 semicélulas 6×22.</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -5560,12 +5560,12 @@
       </c>
       <c r="U67" t="inlineStr">
         <is>
-          <t>Ficha oficial EINNOVA ESM-T series — Ns estimado (confirmar dims)</t>
+          <t>Ficha oficial EINNOVA ESM-T — 132 piezas (6×22) confirmadas</t>
         </is>
       </c>
       <c r="V67" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Ficha oficial EINNOVA ESM-545T TopCon Bifacial. Efic=22.95%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims ESTIMADAS — confirmar con EINNOVA.</t>
+          <t>Ficha oficial EINNOVA ESM-545T TopCon Bifacial. Efic=22.95%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims CONFIRMADAS: 2094×1134×30mm. 132 semicélulas 6×22.</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -5633,12 +5633,12 @@
       </c>
       <c r="U68" t="inlineStr">
         <is>
-          <t>Ficha oficial EINNOVA ESM-T series — Ns estimado (confirmar dims)</t>
+          <t>Ficha oficial EINNOVA ESM-T — 132 piezas (6×22) confirmadas</t>
         </is>
       </c>
       <c r="V68" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>
@@ -5672,7 +5672,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>Ficha oficial EINNOVA ESM-550T TopCon Bifacial. Efic=23.16%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims ESTIMADAS — confirmar con EINNOVA.</t>
+          <t>Ficha oficial EINNOVA ESM-550T TopCon Bifacial. Efic=23.16%. CoefIsc=+0.04%/°C. Vmax=1500Vdc. Dims CONFIRMADAS: 2094×1134×30mm. 132 semicélulas 6×22.</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -5706,12 +5706,12 @@
       </c>
       <c r="U69" t="inlineStr">
         <is>
-          <t>Ficha oficial EINNOVA ESM-T series — Ns estimado (confirmar dims)</t>
+          <t>Ficha oficial EINNOVA ESM-T — 132 piezas (6×22) confirmadas</t>
         </is>
       </c>
       <c r="V69" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: EINNOVA Agri ESM-305HE Bifacial al catálogo (fila 70) — BIPV agri τ=38%
</commit_message>
<xml_diff>
--- a/bipv_python/datos/paneles_catalogo.xlsx
+++ b/bipv_python/datos/paneles_catalogo.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V69"/>
+  <dimension ref="A1:V70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5715,6 +5715,79 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>EINNOVA Solarline</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>EINNOVA Agri ESM-305HE Bifacial</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>305</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>1762x1134x30</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>45</v>
+      </c>
+      <c r="H70" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="I70" t="n">
+        <v>38</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA Agri ESM-305HE. Panel agrícola semitransparente τ=38%. TOPCon N-Type 182×105mm (4×16pcs=64 celdas). Dual glass 2+2mm. Marco: fibra vidrio reforzada con poliuretano. Vmax=1500Vdc. CoefIsc=+0.045%/°C. IEC61215/61730. Agrivoltaico/BIPV.</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>N-Type TopCon Bifacial Agri</t>
+        </is>
+      </c>
+      <c r="L70" t="n">
+        <v>23.65</v>
+      </c>
+      <c r="M70" t="n">
+        <v>20</v>
+      </c>
+      <c r="N70" t="n">
+        <v>15.73</v>
+      </c>
+      <c r="O70" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="P70" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>64</v>
+      </c>
+      <c r="R70" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="S70" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-305HE — 4×16 celdas TOPCon 182×105mm</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
feat: EINNOVA ESM-400 Terra Cotta TopCon al catálogo (fila 71) — BIPV decorativo τ=0%
</commit_message>
<xml_diff>
--- a/bipv_python/datos/paneles_catalogo.xlsx
+++ b/bipv_python/datos/paneles_catalogo.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V70"/>
+  <dimension ref="A1:V71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5788,6 +5788,79 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>EINNOVA Solarline</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>EINNOVA ESM-400 Terra Cotta TopCon</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>400</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>1762x1134x30</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>45</v>
+      </c>
+      <c r="H71" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-400 Terra Cotta. Panel BIPV decorativo con vidrio color terracota — OPACO (τ=0%). TOPCon N-Type Monocristalino. CoefIsc=+0.046%/°C. Tolerancia 0~+3%. Vmax=1500Vdc. Dims y Ns ESTIMADOS (confirmar con EINNOVA). Precio pendiente.</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>N-Type TopCon Mono Colored Glass</t>
+        </is>
+      </c>
+      <c r="L71" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="M71" t="n">
+        <v>33.25</v>
+      </c>
+      <c r="N71" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="O71" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="P71" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>54</v>
+      </c>
+      <c r="R71" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="S71" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>Ficha oficial EINNOVA ESM-400 Terracota — Ns estimado (confirmar con fabricante)</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
fix: ESM-400 Terra Cotta dims confirmadas 1722×1134×30mm, 108 semicél (6×18) N_s=54, Confianza=Alta
</commit_message>
<xml_diff>
--- a/bipv_python/datos/paneles_catalogo.xlsx
+++ b/bipv_python/datos/paneles_catalogo.xlsx
@@ -5804,7 +5804,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>1762x1134x30</t>
+          <t>1722x1134x30</t>
         </is>
       </c>
       <c r="G71" t="n">
@@ -5818,7 +5818,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Ficha oficial EINNOVA ESM-400 Terra Cotta. Panel BIPV decorativo con vidrio color terracota — OPACO (τ=0%). TOPCon N-Type Monocristalino. CoefIsc=+0.046%/°C. Tolerancia 0~+3%. Vmax=1500Vdc. Dims y Ns ESTIMADOS (confirmar con EINNOVA). Precio pendiente.</t>
+          <t>Ficha oficial EINNOVA ESM-400 Terra Cotta. Panel BIPV decorativo vidrio color terracota — OPACO (τ=0%). TOPCon N-Type 182×93.4mm half-cells. 108 piezas (6×18) → N_s=54 en serie. Dims CONFIRMADAS: 1722×1134×30mm. CoefIsc=+0.046%/°C. Vmax=1500Vdc. Precio pendiente.</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -5852,12 +5852,12 @@
       </c>
       <c r="U71" t="inlineStr">
         <is>
-          <t>Ficha oficial EINNOVA ESM-400 Terracota — Ns estimado (confirmar con fabricante)</t>
+          <t>Ficha oficial EINNOVA ESM-400 — 108 semicélulas (6×18) 182×93.4mm → N_s=54 en serie</t>
         </is>
       </c>
       <c r="V71" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: EINNOVA ESM-FT 120W Flat Tile Color (fila 72) — teja solar BIPV doble vidrio τ=0%
</commit_message>
<xml_diff>
--- a/bipv_python/datos/paneles_catalogo.xlsx
+++ b/bipv_python/datos/paneles_catalogo.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V71"/>
+  <dimension ref="A1:V72"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5861,6 +5861,76 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>EINNOVA Solarline</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>EINNOVA ESM-FT 120W Flat Tile Color</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>120</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>1600x460x6</t>
+        </is>
+      </c>
+      <c r="H72" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>EINNOVA ESM-FT 120W — Teja solar plana doble vidrio BIPV. Colores: negro, gris, rojo/terracota. OPACA (τ=0%). Dims CONFIRMADAS: 1600×460×6mm. Peso 13.5kg. Vmax=1000Vdc. Fusible 20A. Efic. 21.8% = eficiencia de celda (módulo=16.3% sobre área total). Ficha STC indica 20°C celda (no estándar — asumido 25°C). CoefT_C y CoefVoc_C ESTIMADOS para N-Type TOPCon. N_s ESTIMADO. Nota: módulo pequeño (120W) — requiere más unidades en serie por string. Precio pendiente.</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>N-Type TOPCon Double Glass BIPV Tile</t>
+        </is>
+      </c>
+      <c r="L72" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="M72" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="N72" t="n">
+        <v>13.26</v>
+      </c>
+      <c r="O72" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="P72" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>15</v>
+      </c>
+      <c r="R72" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="S72" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>N_s ESTIMADO: 10.99V / 0.73V célula TOPCon ≈ 15. Confirmar con EINNOVA</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
feat: agregar 6 modelos JA Solar JAM66D46-LB (715–740W N-Type Bifacial) + filtrar entradas basura del catálogo
</commit_message>
<xml_diff>
--- a/bipv_python/datos/paneles_catalogo.xlsx
+++ b/bipv_python/datos/paneles_catalogo.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V72"/>
+  <dimension ref="A1:V78"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5931,6 +5931,378 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>JA Solar</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>JA Solar JAM66D46-715/LB</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>715</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2384x1303x33 mm</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>45</v>
+      </c>
+      <c r="H73" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>N-Type n-Bycium+ 18BB Half-Cut Double Glass Bifacial. Max sys voltage 1500 VDC. Bifacialidad 80%±5%. 0.4% degradación anual (30 años). NOCT 45±2°C.</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>N-Type TOPCon Bifacial</t>
+        </is>
+      </c>
+      <c r="L73" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="M73" t="n">
+        <v>41</v>
+      </c>
+      <c r="N73" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="O73" t="n">
+        <v>17.44</v>
+      </c>
+      <c r="P73" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>66</v>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>Alta — ficha oficial JA Solar Global-EN-20250709C</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>JA Solar</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>JA Solar JAM66D46-720/LB</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>720</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>2384x1303x33 mm</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>45</v>
+      </c>
+      <c r="H74" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="I74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>N-Type n-Bycium+ 18BB Half-Cut Double Glass Bifacial. Max sys voltage 1500 VDC. Bifacialidad 80%±5%. 0.4% degradación anual (30 años). NOCT 45±2°C.</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>N-Type TOPCon Bifacial</t>
+        </is>
+      </c>
+      <c r="L74" t="n">
+        <v>49</v>
+      </c>
+      <c r="M74" t="n">
+        <v>41.19</v>
+      </c>
+      <c r="N74" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="O74" t="n">
+        <v>17.48</v>
+      </c>
+      <c r="P74" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>66</v>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>Alta — ficha oficial JA Solar Global-EN-20250709C</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>JA Solar</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>JA Solar JAM66D46-725/LB</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>725</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2384x1303x33 mm</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>45</v>
+      </c>
+      <c r="H75" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="I75" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>N-Type n-Bycium+ 18BB Half-Cut Double Glass Bifacial. Max sys voltage 1500 VDC. Bifacialidad 80%±5%. 0.4% degradación anual (30 años). NOCT 45±2°C.</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>N-Type TOPCon Bifacial</t>
+        </is>
+      </c>
+      <c r="L75" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="M75" t="n">
+        <v>41.39</v>
+      </c>
+      <c r="N75" t="n">
+        <v>18.63</v>
+      </c>
+      <c r="O75" t="n">
+        <v>17.52</v>
+      </c>
+      <c r="P75" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>66</v>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>Alta — ficha oficial JA Solar Global-EN-20250709C</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>JA Solar</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>JA Solar JAM66D46-730/LB</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>730</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>2384x1303x33 mm</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>45</v>
+      </c>
+      <c r="H76" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="I76" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>N-Type n-Bycium+ 18BB Half-Cut Double Glass Bifacial. Max sys voltage 1500 VDC. Bifacialidad 80%±5%. 0.4% degradación anual (30 años). NOCT 45±2°C.</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>N-Type TOPCon Bifacial</t>
+        </is>
+      </c>
+      <c r="L76" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="M76" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="N76" t="n">
+        <v>18.67</v>
+      </c>
+      <c r="O76" t="n">
+        <v>17.56</v>
+      </c>
+      <c r="P76" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>66</v>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>Alta — ficha oficial JA Solar Global-EN-20250709C</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>JA Solar</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>JA Solar JAM66D46-735/LB</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>735</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2384x1303x33 mm</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>45</v>
+      </c>
+      <c r="H77" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>N-Type n-Bycium+ 18BB Half-Cut Double Glass Bifacial. Max sys voltage 1500 VDC. Bifacialidad 80%±5%. 0.4% degradación anual (30 años). NOCT 45±2°C.</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>N-Type TOPCon Bifacial</t>
+        </is>
+      </c>
+      <c r="L77" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="M77" t="n">
+        <v>41.77</v>
+      </c>
+      <c r="N77" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="O77" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="P77" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>66</v>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>Alta — ficha oficial JA Solar Global-EN-20250709C</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>JA Solar</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>JA Solar JAM66D46-740/LB</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>740</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>2384x1303x33 mm</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>45</v>
+      </c>
+      <c r="H78" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>N-Type n-Bycium+ 18BB Half-Cut Double Glass Bifacial. Max sys voltage 1500 VDC. Bifacialidad 80%±5%. 0.4% degradación anual (30 años). NOCT 45±2°C.</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>N-Type TOPCon Bifacial</t>
+        </is>
+      </c>
+      <c r="L78" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="M78" t="n">
+        <v>41.96</v>
+      </c>
+      <c r="N78" t="n">
+        <v>18.73</v>
+      </c>
+      <c r="O78" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="P78" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>66</v>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>Alta — ficha oficial JA Solar Global-EN-20250709C</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
fix: corregir Ns=132→66 en Tensite 710W, JAM66D45-625/LB y EINNOVA ESM-620M (half-cut → N_s eléctrico=66)
</commit_message>
<xml_diff>
--- a/bipv_python/datos/paneles_catalogo.xlsx
+++ b/bipv_python/datos/paneles_catalogo.xlsx
@@ -5112,7 +5112,7 @@
         <v>-0.25</v>
       </c>
       <c r="Q61" t="n">
-        <v>132</v>
+        <v>66</v>
       </c>
       <c r="R61" t="n">
         <v>1.3</v>
@@ -5185,7 +5185,7 @@
         <v>-0.25</v>
       </c>
       <c r="Q62" t="n">
-        <v>132</v>
+        <v>66</v>
       </c>
       <c r="R62" t="n">
         <v>1.3</v>
@@ -5331,7 +5331,7 @@
         <v>-0.26</v>
       </c>
       <c r="Q64" t="n">
-        <v>132</v>
+        <v>66</v>
       </c>
       <c r="R64" t="n">
         <v>1.3</v>

</xml_diff>

<commit_message>
feat: simulación bifacial completa con pvlib infinite_sheds — bifacialidad en catálogo, altura/albedo trasero/GCR en Recurso Solar, ganancia integrada al POA y a multi-superficie
</commit_message>
<xml_diff>
--- a/bipv_python/datos/paneles_catalogo.xlsx
+++ b/bipv_python/datos/paneles_catalogo.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Catalogo_Paneles_FV" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo_Paneles_FV" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V78"/>
+  <dimension ref="A1:W78"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -610,6 +610,11 @@
           <t>Confianza</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>BifacialidadPct</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -5992,6 +5997,9 @@
           <t>Alta — ficha oficial JA Solar Global-EN-20250709C</t>
         </is>
       </c>
+      <c r="W73" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="74">
       <c r="B74" t="inlineStr">
@@ -6054,6 +6062,9 @@
           <t>Alta — ficha oficial JA Solar Global-EN-20250709C</t>
         </is>
       </c>
+      <c r="W74" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="75">
       <c r="B75" t="inlineStr">
@@ -6116,6 +6127,9 @@
           <t>Alta — ficha oficial JA Solar Global-EN-20250709C</t>
         </is>
       </c>
+      <c r="W75" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="76">
       <c r="B76" t="inlineStr">
@@ -6178,6 +6192,9 @@
           <t>Alta — ficha oficial JA Solar Global-EN-20250709C</t>
         </is>
       </c>
+      <c r="W76" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="77">
       <c r="B77" t="inlineStr">
@@ -6240,6 +6257,9 @@
           <t>Alta — ficha oficial JA Solar Global-EN-20250709C</t>
         </is>
       </c>
+      <c r="W77" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
@@ -6301,6 +6321,9 @@
         <is>
           <t>Alta — ficha oficial JA Solar Global-EN-20250709C</t>
         </is>
+      </c>
+      <c r="W78" t="n">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>